<commit_message>
CORE-000083 edit: --TESTCD added in output variables and validation sheets updated accordingly
</commit_message>
<xml_diff>
--- a/rules/CORE-000083/negative/01/data/unit-test-coreid-CG0553-negative1.xlsx
+++ b/rules/CORE-000083/negative/01/data/unit-test-coreid-CG0553-negative1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marisa_wyckmans\CORE\CDISC_Rule_Authoring\core-contributor\rules\CORE-000083\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F565DB6-4679-49D8-81D7-D035B858E266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B0075D4-4974-4204-9A0A-4C8640DFDE6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21240" windowHeight="15270" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="81">
   <si>
     <t>Product</t>
   </si>
@@ -747,7 +747,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="16" customWidth="1"/>
@@ -788,7 +788,10 @@
         <v>5</v>
       </c>
       <c r="E2" t="s">
-        <v>21</v>
+        <v>18</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -805,10 +808,7 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F3" t="s">
-        <v>64</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -825,12 +825,15 @@
         <v>5</v>
       </c>
       <c r="E4" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="F4" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
@@ -839,10 +842,10 @@
         <v>71</v>
       </c>
       <c r="D5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -859,10 +862,10 @@
         <v>6</v>
       </c>
       <c r="E6" t="s">
-        <v>28</v>
-      </c>
-      <c r="F6" t="s">
-        <v>64</v>
+        <v>18</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -879,12 +882,12 @@
         <v>6</v>
       </c>
       <c r="E7" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B8" t="s">
         <v>6</v>
@@ -893,15 +896,18 @@
         <v>71</v>
       </c>
       <c r="D8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E8" t="s">
-        <v>21</v>
+        <v>28</v>
+      </c>
+      <c r="F8" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B9" t="s">
         <v>6</v>
@@ -910,13 +916,10 @@
         <v>71</v>
       </c>
       <c r="D9">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E9" t="s">
-        <v>28</v>
-      </c>
-      <c r="F9" t="s">
-        <v>64</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -933,6 +936,63 @@
         <v>7</v>
       </c>
       <c r="E10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" t="s">
+        <v>71</v>
+      </c>
+      <c r="D11">
+        <v>7</v>
+      </c>
+      <c r="E11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s">
+        <v>71</v>
+      </c>
+      <c r="D12">
+        <v>7</v>
+      </c>
+      <c r="E12" t="s">
+        <v>28</v>
+      </c>
+      <c r="F12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13">
+        <v>7</v>
+      </c>
+      <c r="E13" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1219,7 +1279,7 @@
       <c r="D5" s="4">
         <v>3</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>72</v>
       </c>
       <c r="F5" s="4" t="s">
@@ -1276,7 +1336,7 @@
       <c r="D6" s="3">
         <v>18</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="6" t="s">
         <v>67</v>
       </c>
       <c r="F6" s="3" t="s">
@@ -1333,7 +1393,7 @@
       <c r="D7" s="3">
         <v>46</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="6" t="s">
         <v>75</v>
       </c>
       <c r="F7" s="3" t="s">

</xml_diff>